<commit_message>
Add updated long format
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v16_long.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v16_long.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C54162-3261-1E41-A900-519BB4B70E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881ABCE3-607C-974B-9DD8-256DE65F55EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="287">
   <si>
     <t>Field Name</t>
   </si>
@@ -499,9 +499,6 @@
     <t>as in: dried; format: character</t>
   </si>
   <si>
-    <t>Type of sample procudure prior to anlysis (dried, ground)</t>
-  </si>
-  <si>
     <t>source_id (e.g., 1)</t>
   </si>
   <si>
@@ -541,16 +538,10 @@
     <t>as in: Timothy B. Johnson; format: character</t>
   </si>
   <si>
-    <t>Literature soruce id</t>
-  </si>
-  <si>
     <t xml:space="preserve">Type of literature source; Report, Journal Article, Book, Book Section ect. </t>
   </si>
   <si>
     <t>Author names</t>
-  </si>
-  <si>
-    <t>Affilation of corresponding author</t>
   </si>
   <si>
     <t>Email address of corresponding author</t>
@@ -625,9 +616,6 @@
     <t xml:space="preserve">Weight of the sample </t>
   </si>
   <si>
-    <t xml:space="preserve">Converstion factor for calorimetry </t>
-  </si>
-  <si>
     <t xml:space="preserve">as in: 5; format: integer </t>
   </si>
   <si>
@@ -656,9 +644,6 @@
   </si>
   <si>
     <t>Date that the sample was collected</t>
-  </si>
-  <si>
-    <t>Genus and speices of the organism</t>
   </si>
   <si>
     <t xml:space="preserve">Sample origins (e.g., wild or lab) </t>
@@ -746,9 +731,6 @@
   </si>
   <si>
     <t>The slope for energy density equations</t>
-  </si>
-  <si>
-    <t>The y-intercept for engery density equations</t>
   </si>
   <si>
     <t>The units for the x variable in relation to slope and intercept</t>
@@ -868,16 +850,10 @@
     <t>as: Point Petre; format: character</t>
   </si>
   <si>
-    <t xml:space="preserve">as in: 1.35; format: numeric; places 2 decmials </t>
-  </si>
-  <si>
     <t>tbl_length</t>
   </si>
   <si>
     <t>trt_description</t>
-  </si>
-  <si>
-    <t>as in: control: format: character</t>
   </si>
   <si>
     <t>as in: benjamin.hlina@gmail.com - valid email address; format: character</t>
@@ -947,9 +923,6 @@
   </si>
   <si>
     <t xml:space="preserve">Email address of submitting person </t>
-  </si>
-  <si>
-    <t>Affilation of submitting person</t>
   </si>
   <si>
     <t>as in: Benjamin L. Hlina; format: character</t>
@@ -1189,9 +1162,6 @@
     <t xml:space="preserve">Type of Polychlorimated biphenols (PCB) congener </t>
   </si>
   <si>
-    <t>tbl_thamine</t>
-  </si>
-  <si>
     <t>tbl_contaminants</t>
   </si>
   <si>
@@ -1199,6 +1169,33 @@
   </si>
   <si>
     <t>tbl_thiamine</t>
+  </si>
+  <si>
+    <t>Literature source id</t>
+  </si>
+  <si>
+    <t>Affiliation of submitting person</t>
+  </si>
+  <si>
+    <t>Affiliation of corresponding author</t>
+  </si>
+  <si>
+    <t>Genus and species of the organism</t>
+  </si>
+  <si>
+    <t>Type of sample procedure prior to analysis (dried, ground)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as in: 1.35; format: numeric; places 2 decimals </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conversion factor for calorimetry </t>
+  </si>
+  <si>
+    <t>The y-intercept for energy density equations</t>
+  </si>
+  <si>
+    <t>as in: control; format: character</t>
   </si>
 </sst>
 </file>
@@ -1928,7 +1925,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="52" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B1" s="52"/>
       <c r="C1" s="52"/>
@@ -1936,7 +1933,7 @@
     </row>
     <row r="2" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="52" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="B2" s="52"/>
       <c r="C2" s="52"/>
@@ -1958,49 +1955,49 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="56" x14ac:dyDescent="0.2">
       <c r="A7" s="29" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>218</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="32" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B8" s="33" t="s">
         <v>4</v>
@@ -2009,214 +2006,214 @@
         <v>66</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>94</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A9" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B10" s="34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="56" x14ac:dyDescent="0.2">
       <c r="A11" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>97</v>
+        <v>280</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B12" s="34" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="D12" s="31" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B14" s="34" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D18" s="31" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D19" s="31" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B21" s="31" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B22" s="31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D22" s="31" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="35" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B23" s="36" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D23" s="27" t="s">
         <v>18</v>
@@ -2224,10 +2221,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C24" s="37" t="s">
         <v>40</v>
@@ -2238,69 +2235,69 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B25" s="38" t="s">
         <v>70</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B26" s="37" t="s">
         <v>5</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B27" s="37" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C27" s="37" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="D27" s="37" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C28" s="37" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D28" s="37" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B29" s="37" t="s">
         <v>6</v>
       </c>
       <c r="C29" s="37" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D29" s="37" t="s">
         <v>11</v>
@@ -2308,55 +2305,55 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B30" s="39" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="C30" s="37" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>133</v>
+        <v>281</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B31" s="37" t="s">
         <v>15</v>
       </c>
       <c r="C31" s="37" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D31" s="37" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B32" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="C32" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="D32" s="37" t="s">
         <v>127</v>
-      </c>
-      <c r="C32" s="37" t="s">
-        <v>168</v>
-      </c>
-      <c r="D32" s="37" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B33" s="37" t="s">
         <v>7</v>
       </c>
       <c r="C33" s="37" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D33" s="37" t="s">
         <v>41</v>
@@ -2364,21 +2361,21 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B34" s="37" t="s">
         <v>8</v>
       </c>
       <c r="C34" s="37" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="D34" s="37" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B35" s="39" t="s">
         <v>13</v>
@@ -2387,29 +2384,29 @@
         <v>50</v>
       </c>
       <c r="D35" s="40" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A36" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B36" s="37" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C36" s="37" t="s">
-        <v>194</v>
+        <v>286</v>
       </c>
       <c r="D36" s="40" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B37" s="37" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C37" s="37" t="s">
         <v>49</v>
@@ -2420,49 +2417,49 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="37" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="B38" s="37" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C38" s="37" t="s">
         <v>51</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A39" s="37" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="B39" s="37" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C39" s="37" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="D39" s="40" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B40" s="37" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="C40" s="37" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D40" s="37" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B41" s="37" t="s">
         <v>72</v>
@@ -2471,12 +2468,12 @@
         <v>74</v>
       </c>
       <c r="D41" s="37" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B42" s="37" t="s">
         <v>73</v>
@@ -2490,7 +2487,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B43" s="39" t="s">
         <v>9</v>
@@ -2504,7 +2501,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B44" s="39" t="s">
         <v>78</v>
@@ -2513,7 +2510,7 @@
         <v>79</v>
       </c>
       <c r="D44" s="37" t="s">
-        <v>80</v>
+        <v>282</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
@@ -2521,13 +2518,13 @@
         <v>16</v>
       </c>
       <c r="B45" s="37" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C45" s="37" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D45" s="37" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
@@ -2552,10 +2549,10 @@
         <v>19</v>
       </c>
       <c r="C47" s="37" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D47" s="37" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
@@ -2569,7 +2566,7 @@
         <v>60</v>
       </c>
       <c r="D48" s="37" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
@@ -2580,7 +2577,7 @@
         <v>21</v>
       </c>
       <c r="C49" s="37" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D49" s="37" t="s">
         <v>61</v>
@@ -2594,7 +2591,7 @@
         <v>22</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>26</v>
@@ -2608,10 +2605,10 @@
         <v>23</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
@@ -2633,13 +2630,13 @@
         <v>28</v>
       </c>
       <c r="B53" s="41" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>191</v>
+        <v>283</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>122</v>
+        <v>284</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
@@ -2647,13 +2644,13 @@
         <v>28</v>
       </c>
       <c r="B54" s="37" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="C54" s="37" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D54" s="37" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
@@ -2661,13 +2658,13 @@
         <v>28</v>
       </c>
       <c r="B55" s="37" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C55" s="37" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D55" s="37" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
@@ -2675,13 +2672,13 @@
         <v>28</v>
       </c>
       <c r="B56" s="37" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C56" s="37" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D56" s="37" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
@@ -2689,13 +2686,13 @@
         <v>28</v>
       </c>
       <c r="B57" s="42" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C57" s="37" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D57" s="37" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
@@ -2703,13 +2700,13 @@
         <v>28</v>
       </c>
       <c r="B58" s="37" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C58" s="37" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D58" s="37" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
@@ -2717,13 +2714,13 @@
         <v>28</v>
       </c>
       <c r="B59" s="37" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C59" s="37" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="D59" s="37" t="s">
-        <v>151</v>
+        <v>285</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
@@ -2731,13 +2728,13 @@
         <v>28</v>
       </c>
       <c r="B60" s="42" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C60" s="37" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D60" s="37" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
@@ -2745,13 +2742,13 @@
         <v>28</v>
       </c>
       <c r="B61" s="42" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C61" s="37" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D61" s="37" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
@@ -2885,13 +2882,13 @@
         <v>39</v>
       </c>
       <c r="B71" s="37" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="C71" s="37" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="D71" s="37" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -2899,13 +2896,13 @@
         <v>39</v>
       </c>
       <c r="B72" s="37" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="C72" s="37" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="D72" s="37" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -2913,223 +2910,223 @@
         <v>39</v>
       </c>
       <c r="B73" s="37" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C73" s="37" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D73" s="37" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="B74" s="43" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="29" x14ac:dyDescent="0.2">
       <c r="A75" s="44" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="B75" s="44" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="C75" s="44" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="D75" s="44" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" s="44" t="s">
+        <v>228</v>
+      </c>
+      <c r="B76" s="44" t="s">
+        <v>235</v>
+      </c>
+      <c r="C76" s="44" t="s">
+        <v>236</v>
+      </c>
+      <c r="D76" s="44" t="s">
         <v>237</v>
-      </c>
-      <c r="B76" s="44" t="s">
-        <v>244</v>
-      </c>
-      <c r="C76" s="44" t="s">
-        <v>245</v>
-      </c>
-      <c r="D76" s="44" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="29" x14ac:dyDescent="0.2">
       <c r="A77" s="44" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="B77" s="45" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="C77" s="44" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="D77" s="44" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="43" x14ac:dyDescent="0.2">
       <c r="A78" s="44" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="B78" s="45" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="C78" s="44" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="D78" s="44" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" s="46" t="s">
+        <v>238</v>
+      </c>
+      <c r="B79" s="42" t="s">
+        <v>245</v>
+      </c>
+      <c r="C79" s="46" t="s">
+        <v>246</v>
+      </c>
+      <c r="D79" s="46" t="s">
         <v>247</v>
-      </c>
-      <c r="B79" s="42" t="s">
-        <v>254</v>
-      </c>
-      <c r="C79" s="46" t="s">
-        <v>255</v>
-      </c>
-      <c r="D79" s="46" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" s="46" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="B80" s="37" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="C80" s="46" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="D80" s="44" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="43" x14ac:dyDescent="0.2">
       <c r="A81" s="46" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="B81" s="37" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="C81" s="46" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="D81" s="44" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" s="46" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="B82" s="37" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="C82" s="46" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="D82" s="44" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="46" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="B83" s="37" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="C83" s="46" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="D83" s="46" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" s="46" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="B84" s="37" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="C84" s="46" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="D84" s="46" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" s="46" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="B85" s="37" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="C85" s="46" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="D85" s="46" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="46" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="B86" s="37" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="C86" s="46" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="D86" s="46" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" s="46" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="B87" s="37" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="C87" s="46" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="D87" s="46" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" s="46" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="B88" s="37" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="C88" s="46" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="D88" s="46" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -3153,12 +3150,12 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="B1" s="54"/>
       <c r="C1" s="54"/>
       <c r="D1" s="16" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -3174,18 +3171,18 @@
       <c r="B3" s="53"/>
       <c r="C3" s="53"/>
       <c r="D3" s="17" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="20" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -3219,12 +3216,12 @@
   <sheetData>
     <row r="1" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="B1" s="54"/>
       <c r="C1" s="54"/>
       <c r="D1" s="16" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -3245,49 +3242,49 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="22" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="B4" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="F4" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G4" s="23" t="s">
-        <v>137</v>
-      </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="K4" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="O4" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
@@ -44244,12 +44241,12 @@
   <sheetData>
     <row r="1" spans="1:68" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B1" s="54"/>
       <c r="C1" s="54"/>
       <c r="D1" s="5" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:68" x14ac:dyDescent="0.2">
@@ -44270,7 +44267,7 @@
     </row>
     <row r="4" spans="1:68" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="X4" t="s">
         <v>16</v>
@@ -44285,25 +44282,25 @@
         <v>39</v>
       </c>
       <c r="BB4" s="47" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="BC4" s="47"/>
       <c r="BD4" s="47"/>
       <c r="BE4" s="47" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="BF4" s="47"/>
       <c r="BG4" s="47"/>
       <c r="BH4" s="47" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="BI4" s="48"/>
       <c r="BJ4" s="48"/>
       <c r="BK4" s="48" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="BL4" s="48" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="BM4" s="48"/>
       <c r="BN4" s="48"/>
@@ -44315,37 +44312,37 @@
         <v>14</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>65</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>15</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="M5" s="12" t="s">
         <v>8</v>
@@ -44354,19 +44351,19 @@
         <v>13</v>
       </c>
       <c r="O5" s="12" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="P5" s="12" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="Q5" s="12" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="R5" s="12" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="T5" s="13" t="s">
         <v>72</v>
@@ -44381,7 +44378,7 @@
         <v>71</v>
       </c>
       <c r="X5" s="13" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="Y5" s="11" t="s">
         <v>17</v>
@@ -44396,40 +44393,40 @@
         <v>21</v>
       </c>
       <c r="AC5" s="15" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="AD5" s="15" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="AE5" s="15" t="s">
         <v>67</v>
       </c>
       <c r="AF5" s="15" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="AG5" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="AH5" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI5" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="AJ5" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="AK5" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="AL5" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="AM5" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="AH5" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="AI5" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="AJ5" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="AK5" s="13" t="s">
+      <c r="AN5" s="13" t="s">
         <v>144</v>
-      </c>
-      <c r="AL5" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="AM5" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="AN5" s="13" t="s">
-        <v>149</v>
       </c>
       <c r="AO5" s="12" t="s">
         <v>29</v>
@@ -44450,7 +44447,7 @@
         <v>35</v>
       </c>
       <c r="AU5" s="12" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="AV5" s="12" t="s">
         <v>36</v>
@@ -44462,58 +44459,58 @@
         <v>38</v>
       </c>
       <c r="AY5" s="12" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="AZ5" s="12" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="BA5" s="12" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="BB5" s="49" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="BC5" s="50" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="BD5" s="50" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="BE5" s="51" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="BF5" s="51" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="BG5" s="51" t="s">
+        <v>245</v>
+      </c>
+      <c r="BH5" s="50" t="s">
+        <v>249</v>
+      </c>
+      <c r="BI5" s="50" t="s">
+        <v>252</v>
+      </c>
+      <c r="BJ5" s="50" t="s">
         <v>254</v>
       </c>
-      <c r="BH5" s="50" t="s">
-        <v>258</v>
-      </c>
-      <c r="BI5" s="50" t="s">
-        <v>261</v>
-      </c>
-      <c r="BJ5" s="50" t="s">
+      <c r="BK5" s="50" t="s">
+        <v>257</v>
+      </c>
+      <c r="BL5" s="50" t="s">
+        <v>260</v>
+      </c>
+      <c r="BM5" s="50" t="s">
         <v>263</v>
       </c>
-      <c r="BK5" s="50" t="s">
-        <v>266</v>
-      </c>
-      <c r="BL5" s="50" t="s">
+      <c r="BN5" s="50" t="s">
+        <v>276</v>
+      </c>
+      <c r="BO5" s="50" t="s">
         <v>269</v>
       </c>
-      <c r="BM5" s="50" t="s">
+      <c r="BP5" s="50" t="s">
         <v>272</v>
-      </c>
-      <c r="BN5" s="50" t="s">
-        <v>286</v>
-      </c>
-      <c r="BO5" s="50" t="s">
-        <v>278</v>
-      </c>
-      <c r="BP5" s="50" t="s">
-        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>